<commit_message>
M04 alimentation deterministe sans Power Query - URL centralisee REF
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot6b_DeclarationsInternes/MASTER_NORM_Declarations_Internes.xlsx
+++ b/02_TRAVAIL/Lot6b_DeclarationsInternes/MASTER_NORM_Declarations_Internes.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,30 +488,35 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>cout_lavage_attribue</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>lavage_non_attribuable_mois</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>statut_controle</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>code_controle</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>commentaire</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>date_extraction</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>ROW_HASH</t>
         </is>
@@ -574,24 +579,29 @@
       <c r="L2" t="n">
         <v>20</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" t="n">
+        <v>40</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>412a76157796c535</t>
         </is>
@@ -654,24 +664,29 @@
       <c r="L3" t="n">
         <v>6</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" t="n">
+        <v>13</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>10fe24845310699b</t>
         </is>
@@ -734,24 +749,29 @@
       <c r="L4" t="n">
         <v>8</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>cd99c4ebea0ad575</t>
         </is>
@@ -814,24 +834,29 @@
       <c r="L5" t="n">
         <v>24</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M5" t="n">
+        <v>70</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>fdc6efca63ff5d45</t>
         </is>
@@ -894,24 +919,29 @@
       <c r="L6" t="n">
         <v>25</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M6" t="n">
+        <v>64</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>67ea9a859d63810e</t>
         </is>
@@ -974,24 +1004,29 @@
       <c r="L7" t="n">
         <v>18</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M7" t="n">
+        <v>60</v>
+      </c>
+      <c r="N7" t="n">
+        <v>110</v>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R7" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
         <is>
           <t>86d918eabec2ad65</t>
         </is>
@@ -1054,24 +1089,29 @@
       <c r="L8" t="n">
         <v>15</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M8" t="n">
+        <v>50</v>
+      </c>
+      <c r="N8" t="n">
+        <v>110</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R8" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
         <is>
           <t>cb042425a5d3261c</t>
         </is>
@@ -1134,24 +1174,29 @@
       <c r="L9" t="n">
         <v>3</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M9" t="n">
+        <v>10</v>
+      </c>
+      <c r="N9" t="n">
+        <v>110</v>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R9" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
         <is>
           <t>70877dd74a01ae66</t>
         </is>
@@ -1214,24 +1259,29 @@
       <c r="L10" t="n">
         <v>28</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M10" t="n">
+        <v>80</v>
+      </c>
+      <c r="N10" t="n">
+        <v>110</v>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
         <is>
           <t>3f65a1e12ee25da3</t>
         </is>
@@ -1294,24 +1344,29 @@
       <c r="L11" t="n">
         <v>3</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M11" t="n">
+        <v>10</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R11" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>df44e2430ab62ba1</t>
         </is>
@@ -1374,24 +1429,29 @@
       <c r="L12" t="n">
         <v>4</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M12" t="n">
+        <v>8</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R12" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
         <is>
           <t>34d6b9535638fb15</t>
         </is>
@@ -1454,24 +1514,29 @@
       <c r="L13" t="n">
         <v>9</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M13" t="n">
+        <v>25</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R13" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
         <is>
           <t>042de8d6d554973f</t>
         </is>
@@ -1534,24 +1599,29 @@
       <c r="L14" t="n">
         <v>26</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M14" t="n">
+        <v>51</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R14" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
         <is>
           <t>c73eb58dc740ec04</t>
         </is>
@@ -1614,24 +1684,29 @@
       <c r="L15" t="n">
         <v>11</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M15" t="n">
+        <v>40</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R15" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
         <is>
           <t>7bd60d4dec036460</t>
         </is>
@@ -1694,24 +1769,29 @@
       <c r="L16" t="n">
         <v>31</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="M16" t="n">
+        <v>90</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R16" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
         <is>
           <t>fd2b6b839bff2bc2</t>
         </is>
@@ -1774,24 +1854,29 @@
       <c r="L17" t="n">
         <v>16</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="M17" t="n">
+        <v>60</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R17" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
         <is>
           <t>503757d156fb07a0</t>
         </is>
@@ -1854,24 +1939,29 @@
       <c r="L18" t="n">
         <v>21</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M18" t="n">
+        <v>72</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
         <is>
           <t>2ffecaf01dbc8374</t>
         </is>
@@ -1934,24 +2024,29 @@
       <c r="L19" t="n">
         <v>17.5</v>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="M19" t="n">
+        <v>45</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R19" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
         <is>
           <t>d37f34810f1ff454</t>
         </is>
@@ -2011,24 +2106,29 @@
       <c r="K20" t="n">
         <v>3</v>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R20" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
         <is>
           <t>c6135d3ffa0f8eb8</t>
         </is>
@@ -2088,24 +2188,29 @@
       <c r="K21" t="n">
         <v>1</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>https://docs.google.com/spreadsheets/d/e/2PACX-1vTYNAYa4WcY-ask9viQHJT-wQMwyxkKpoDZGpjrnqqtCzXC1xR_6DnZ0oSVTv5LkQTdqPcfaD1PtdAt/pub?output=csv</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>2026-06-18T10:02:26</t>
-        </is>
-      </c>
       <c r="R21" t="inlineStr">
+        <is>
+          <t>2026-06-18T11:22:24</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
         <is>
           <t>df40be8224d307c7</t>
         </is>

</xml_diff>